<commit_message>
Expand Rentora QA suite: search matrix, validation & boundary tests, reports
Add SearchActions and data-driven test matrices (search, form-validation,
boundary/equivalence), expand testcases, refresh report generation, and
include bug/recommendation reports plus evidence screenshots.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/Rentora-Testcases.xlsx
+++ b/excel/Rentora-Testcases.xlsx
@@ -10,6 +10,9 @@
     <sheet name="AdminPortal" sheetId="5" r:id="rId5"/>
     <sheet name="AccessControl" sheetId="6" r:id="rId6"/>
     <sheet name="Security" sheetId="7" r:id="rId7"/>
+    <sheet name="BoundaryEquivalence" sheetId="8" r:id="rId8"/>
+    <sheet name="SearchMatrix" sheetId="9" r:id="rId9"/>
+    <sheet name="FormValidation" sheetId="10" r:id="rId10"/>
   </sheets>
 </workbook>
 </file>
@@ -830,6 +833,712 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H24"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="42.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="36.83203125" customWidth="1"/>
+    <col min="5" max="5" width="48.83203125" customWidth="1"/>
+    <col min="6" max="6" width="46.83203125" customWidth="1"/>
+    <col min="7" max="7" width="40.83203125" customWidth="1"/>
+    <col min="8" max="8" width="26.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Title</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Precondition</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Description</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Steps</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Expected Result</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Actual Result</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Comments</v>
+      </c>
+    </row>
+    <row r="2" xml:space="preserve">
+      <c r="A2" t="str">
+        <v>FV-01</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Register — Empty full name</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Guest on /register; every field valid except the one under test</v>
+      </c>
+      <c r="D2" t="str">
+        <v>VALIDATION — register input: Empty full name</v>
+      </c>
+      <c r="E2" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /register
+2. Fill an otherwise-valid form
+3. Set the field under test (Empty full name)
+4. Click Create account</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Validation rejects the input; account not created; stays on /register; no HTTP 500</v>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v>Medium | validation | automated</v>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
+      <c r="A3" t="str">
+        <v>FV-02</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Register — Name 300 characters (over-long)</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Guest on /register; every field valid except the one under test</v>
+      </c>
+      <c r="D3" t="str">
+        <v>BVA — register input: Name 300 characters (over-long)</v>
+      </c>
+      <c r="E3" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /register
+2. Fill an otherwise-valid form
+3. Set the field under test (Name 300 characters (over-long))
+4. Click Create account</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Validation rejects the input; account not created; stays on /register; no HTTP 500</v>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
+      <c r="A4" t="str">
+        <v>FV-03</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Register — Email missing @ ('plainaddress')</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Guest on /register; every field valid except the one under test</v>
+      </c>
+      <c r="D4" t="str">
+        <v>EP — register input: Email missing @ ('plainaddress')</v>
+      </c>
+      <c r="E4" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /register
+2. Fill an otherwise-valid form
+3. Set the field under test (Email missing @ ('plainaddress'))
+4. Click Create account</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Validation rejects the input; account not created; stays on /register; no HTTP 500</v>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v>Medium | ep | automated</v>
+      </c>
+    </row>
+    <row r="5" xml:space="preserve">
+      <c r="A5" t="str">
+        <v>FV-04</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Register — Email missing domain ('user@')</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Guest on /register; every field valid except the one under test</v>
+      </c>
+      <c r="D5" t="str">
+        <v>EP — register input: Email missing domain ('user@')</v>
+      </c>
+      <c r="E5" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /register
+2. Fill an otherwise-valid form
+3. Set the field under test (Email missing domain ('user@'))
+4. Click Create account</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Validation rejects the input; account not created; stays on /register; no HTTP 500</v>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v>Medium | ep | automated</v>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6" t="str">
+        <v>FV-05</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Register — Email missing local part ('@domain.com')</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Guest on /register; every field valid except the one under test</v>
+      </c>
+      <c r="D6" t="str">
+        <v>EP — register input: Email missing local part ('@domain.com')</v>
+      </c>
+      <c r="E6" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /register
+2. Fill an otherwise-valid form
+3. Set the field under test (Email missing local part ('@domain.com'))
+4. Click Create account</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Validation rejects the input; account not created; stays on /register; no HTTP 500</v>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v>Medium | ep | automated</v>
+      </c>
+    </row>
+    <row r="7" xml:space="preserve">
+      <c r="A7" t="str">
+        <v>FV-06</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Register — Email with spaces ('a b@x.com')</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Guest on /register; every field valid except the one under test</v>
+      </c>
+      <c r="D7" t="str">
+        <v>EP — register input: Email with spaces ('a b@x.com')</v>
+      </c>
+      <c r="E7" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /register
+2. Fill an otherwise-valid form
+3. Set the field under test (Email with spaces ('a b@x.com'))
+4. Click Create account</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Validation rejects the input; account not created; stays on /register; no HTTP 500</v>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v>Medium | ep | automated</v>
+      </c>
+    </row>
+    <row r="8" xml:space="preserve">
+      <c r="A8" t="str">
+        <v>FV-07</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Register — Email double-@ ('a@@b.com')</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Guest on /register; every field valid except the one under test</v>
+      </c>
+      <c r="D8" t="str">
+        <v>EP — register input: Email double-@ ('a@@b.com')</v>
+      </c>
+      <c r="E8" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /register
+2. Fill an otherwise-valid form
+3. Set the field under test (Email double-@ ('a@@b.com'))
+4. Click Create account</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Validation rejects the input; account not created; stays on /register; no HTTP 500</v>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <v>Medium | ep | automated</v>
+      </c>
+    </row>
+    <row r="9" xml:space="preserve">
+      <c r="A9" t="str">
+        <v>FV-08</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Register — Phone 10 digits (one short)</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Guest on /register; every field valid except the one under test</v>
+      </c>
+      <c r="D9" t="str">
+        <v>BVA — register input: Phone 10 digits (one short)</v>
+      </c>
+      <c r="E9" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /register
+2. Fill an otherwise-valid form
+3. Set the field under test (Phone 10 digits (one short))
+4. Click Create account</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Validation rejects the input; account not created; stays on /register; no HTTP 500</v>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="10" xml:space="preserve">
+      <c r="A10" t="str">
+        <v>FV-09</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Register — Phone 12 digits (one long)</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Guest on /register; every field valid except the one under test</v>
+      </c>
+      <c r="D10" t="str">
+        <v>BVA — register input: Phone 12 digits (one long)</v>
+      </c>
+      <c r="E10" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /register
+2. Fill an otherwise-valid form
+3. Set the field under test (Phone 12 digits (one long))
+4. Click Create account</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Validation rejects the input; account not created; stays on /register; no HTTP 500</v>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="11" xml:space="preserve">
+      <c r="A11" t="str">
+        <v>FV-10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Register — Phone without leading 0 ('1712345678')</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Guest on /register; every field valid except the one under test</v>
+      </c>
+      <c r="D11" t="str">
+        <v>EP — register input: Phone without leading 0 ('1712345678')</v>
+      </c>
+      <c r="E11" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /register
+2. Fill an otherwise-valid form
+3. Set the field under test (Phone without leading 0 ('1712345678'))
+4. Click Create account</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Validation rejects the input; account not created; stays on /register; no HTTP 500</v>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11" t="str">
+        <v>Medium | ep | automated</v>
+      </c>
+    </row>
+    <row r="12" xml:space="preserve">
+      <c r="A12" t="str">
+        <v>FV-11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Register — Phone alphabetic</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Guest on /register; every field valid except the one under test</v>
+      </c>
+      <c r="D12" t="str">
+        <v>EP — register input: Phone alphabetic</v>
+      </c>
+      <c r="E12" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /register
+2. Fill an otherwise-valid form
+3. Set the field under test (Phone alphabetic)
+4. Click Create account</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Validation rejects the input; account not created; stays on /register; no HTTP 500</v>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12" t="str">
+        <v>Medium | ep | automated</v>
+      </c>
+    </row>
+    <row r="13" xml:space="preserve">
+      <c r="A13" t="str">
+        <v>FV-12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Register — Password 6 chars (below min)</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Guest on /register; every field valid except the one under test</v>
+      </c>
+      <c r="D13" t="str">
+        <v>BVA — register input: Password 6 chars (below min)</v>
+      </c>
+      <c r="E13" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /register
+2. Fill an otherwise-valid form
+3. Set the field under test (Password 6 chars (below min))
+4. Click Create account</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Validation rejects the input; account not created; stays on /register; no HTTP 500</v>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="14" xml:space="preserve">
+      <c r="A14" t="str">
+        <v>FV-13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Register — Password empty</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Guest on /register; every field valid except the one under test</v>
+      </c>
+      <c r="D14" t="str">
+        <v>BVA — register input: Password empty</v>
+      </c>
+      <c r="E14" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /register
+2. Fill an otherwise-valid form
+3. Set the field under test (Password empty)
+4. Click Create account</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Validation rejects the input; account not created; stays on /register; no HTTP 500</v>
+      </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
+      <c r="H14" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="15" xml:space="preserve">
+      <c r="A15" t="str">
+        <v>FV-14</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Register — Password/confirm mismatch</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Guest on /register; every field valid except the one under test</v>
+      </c>
+      <c r="D15" t="str">
+        <v>NEGATIVE — register input: Password/confirm mismatch</v>
+      </c>
+      <c r="E15" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /register
+2. Fill an otherwise-valid form
+3. Set the field under test (Password/confirm mismatch)
+4. Click Create account</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Validation rejects the input; account not created; stays on /register; no HTTP 500</v>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
+      <c r="H15" t="str">
+        <v>Medium | negative | automated</v>
+      </c>
+    </row>
+    <row r="16" xml:space="preserve">
+      <c r="A16" t="str">
+        <v>FV-15</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Register — Terms unaccepted</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Guest on /register; every field valid except the one under test</v>
+      </c>
+      <c r="D16" t="str">
+        <v>VALIDATION — register input: Terms unaccepted</v>
+      </c>
+      <c r="E16" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /register
+2. Fill an otherwise-valid form
+3. Set the field under test (Terms unaccepted)
+4. Click Create account</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Validation rejects the input; account not created; stays on /register; no HTTP 500</v>
+      </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
+      <c r="H16" t="str">
+        <v>Medium | validation | automated</v>
+      </c>
+    </row>
+    <row r="17" xml:space="preserve">
+      <c r="A17" t="str">
+        <v>FV-16</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Login — Empty email and password</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Guest on /login</v>
+      </c>
+      <c r="D17" t="str">
+        <v>VALIDATION — login input: Empty email and password</v>
+      </c>
+      <c r="E17" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /login
+2. Enter the credentials under test (Empty email and password)
+3. Click Sign in</v>
+      </c>
+      <c r="F17" t="str">
+        <v>Login denied; stays on /login; no server error</v>
+      </c>
+      <c r="G17" t="str">
+        <v/>
+      </c>
+      <c r="H17" t="str">
+        <v>Medium | validation | automated</v>
+      </c>
+    </row>
+    <row r="18" xml:space="preserve">
+      <c r="A18" t="str">
+        <v>FV-17</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Login — Empty password</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Guest on /login</v>
+      </c>
+      <c r="D18" t="str">
+        <v>VALIDATION — login input: Empty password</v>
+      </c>
+      <c r="E18" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /login
+2. Enter the credentials under test (Empty password)
+3. Click Sign in</v>
+      </c>
+      <c r="F18" t="str">
+        <v>Login denied; stays on /login; no server error</v>
+      </c>
+      <c r="G18" t="str">
+        <v/>
+      </c>
+      <c r="H18" t="str">
+        <v>Medium | validation | automated</v>
+      </c>
+    </row>
+    <row r="19" xml:space="preserve">
+      <c r="A19" t="str">
+        <v>FV-18</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Login — Empty email</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Guest on /login</v>
+      </c>
+      <c r="D19" t="str">
+        <v>VALIDATION — login input: Empty email</v>
+      </c>
+      <c r="E19" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /login
+2. Enter the credentials under test (Empty email)
+3. Click Sign in</v>
+      </c>
+      <c r="F19" t="str">
+        <v>Login denied; stays on /login; no server error</v>
+      </c>
+      <c r="G19" t="str">
+        <v/>
+      </c>
+      <c r="H19" t="str">
+        <v>Medium | validation | automated</v>
+      </c>
+    </row>
+    <row r="20" xml:space="preserve">
+      <c r="A20" t="str">
+        <v>FV-19</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Login — Invalid email format</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Guest on /login</v>
+      </c>
+      <c r="D20" t="str">
+        <v>EP — login input: Invalid email format</v>
+      </c>
+      <c r="E20" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /login
+2. Enter the credentials under test (Invalid email format)
+3. Click Sign in</v>
+      </c>
+      <c r="F20" t="str">
+        <v>Login denied; stays on /login; no server error</v>
+      </c>
+      <c r="G20" t="str">
+        <v/>
+      </c>
+      <c r="H20" t="str">
+        <v>Medium | ep | automated</v>
+      </c>
+    </row>
+    <row r="21" xml:space="preserve">
+      <c r="A21" t="str">
+        <v>FV-20</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Login — Valid email, wrong password</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Guest on /login</v>
+      </c>
+      <c r="D21" t="str">
+        <v>NEGATIVE — login input: Valid email, wrong password</v>
+      </c>
+      <c r="E21" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /login
+2. Enter the credentials under test (Valid email, wrong password)
+3. Click Sign in</v>
+      </c>
+      <c r="F21" t="str">
+        <v>Login denied; stays on /login; no server error</v>
+      </c>
+      <c r="G21" t="str">
+        <v/>
+      </c>
+      <c r="H21" t="str">
+        <v>Medium | negative | automated</v>
+      </c>
+    </row>
+    <row r="22" xml:space="preserve">
+      <c r="A22" t="str">
+        <v>FV-21</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Login — Non-existent account</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Guest on /login</v>
+      </c>
+      <c r="D22" t="str">
+        <v>NEGATIVE — login input: Non-existent account</v>
+      </c>
+      <c r="E22" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /login
+2. Enter the credentials under test (Non-existent account)
+3. Click Sign in</v>
+      </c>
+      <c r="F22" t="str">
+        <v>Login denied; stays on /login; no server error</v>
+      </c>
+      <c r="G22" t="str">
+        <v/>
+      </c>
+      <c r="H22" t="str">
+        <v>Medium | negative | automated</v>
+      </c>
+    </row>
+    <row r="23" xml:space="preserve">
+      <c r="A23" t="str">
+        <v>FV-22</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Login — SQL-injection string in email</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Guest on /login</v>
+      </c>
+      <c r="D23" t="str">
+        <v>SECURITY — login input: SQL-injection string in email</v>
+      </c>
+      <c r="E23" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /login
+2. Enter the credentials under test (SQL-injection string in email)
+3. Click Sign in</v>
+      </c>
+      <c r="F23" t="str">
+        <v>Login denied; stays on /login; no server error</v>
+      </c>
+      <c r="G23" t="str">
+        <v/>
+      </c>
+      <c r="H23" t="str">
+        <v>High | security | automated</v>
+      </c>
+    </row>
+    <row r="24" xml:space="preserve">
+      <c r="A24" t="str">
+        <v>FV-23</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Login — Over-long credentials (500 chars)</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Guest on /login</v>
+      </c>
+      <c r="D24" t="str">
+        <v>BVA — login input: Over-long credentials (500 chars)</v>
+      </c>
+      <c r="E24" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /login
+2. Enter the credentials under test (Over-long credentials (500 chars))
+3. Click Sign in</v>
+      </c>
+      <c r="F24" t="str">
+        <v>Login denied; stays on /login; no server error</v>
+      </c>
+      <c r="G24" t="str">
+        <v/>
+      </c>
+      <c r="H24" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H24"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H12"/>
@@ -2281,4 +2990,2831 @@
     <ignoredError numberStoredAsText="1" sqref="A1:H6"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H22"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="42.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="36.83203125" customWidth="1"/>
+    <col min="5" max="5" width="48.83203125" customWidth="1"/>
+    <col min="6" max="6" width="46.83203125" customWidth="1"/>
+    <col min="7" max="7" width="40.83203125" customWidth="1"/>
+    <col min="8" max="8" width="26.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Title</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Precondition</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Description</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Steps</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Expected Result</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Actual Result</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Comments</v>
+      </c>
+    </row>
+    <row r="2" xml:space="preserve">
+      <c r="A2" t="str">
+        <v>BVA-01</v>
+      </c>
+      <c r="B2" t="str">
+        <v>min_price on the lower boundary keeps the cheapest listing (৳6,000)</v>
+      </c>
+      <c r="C2" t="str">
+        <v>8 approved listings; lowest rent = ৳6,000</v>
+      </c>
+      <c r="D2" t="str">
+        <v>BVA — exact lower boundary; min_price equal to the cheapest rent must include it</v>
+      </c>
+      <c r="E2" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?min_price=6000
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F2" t="str">
+        <v>8 rentals found (rent&gt;=6000 is inclusive, the ৳6,000 listing is retained)</v>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v>High | bva | automated</v>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
+      <c r="A3" t="str">
+        <v>BVA-02</v>
+      </c>
+      <c r="B3" t="str">
+        <v>min_price one above the lower boundary drops the cheapest listing</v>
+      </c>
+      <c r="C3" t="str">
+        <v>8 approved listings; lowest rent = ৳6,000</v>
+      </c>
+      <c r="D3" t="str">
+        <v>BVA — boundary+1; min_price = 6001 must exclude the ৳6,000 listing</v>
+      </c>
+      <c r="E3" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?min_price=6001
+2. Read the result counter</v>
+      </c>
+      <c r="F3" t="str">
+        <v>7 rentals found (only the ৳6,000 listing is excluded)</v>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v>High | bva | automated</v>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
+      <c r="A4" t="str">
+        <v>BVA-03</v>
+      </c>
+      <c r="B4" t="str">
+        <v>min_price on the upper boundary keeps only the most expensive listing</v>
+      </c>
+      <c r="C4" t="str">
+        <v>8 approved listings; highest rent = ৳35,000</v>
+      </c>
+      <c r="D4" t="str">
+        <v>BVA — exact upper boundary; min_price equal to the dearest rent keeps just that one</v>
+      </c>
+      <c r="E4" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?min_price=35000
+2. Read the result counter</v>
+      </c>
+      <c r="F4" t="str">
+        <v>1 rental found (only the ৳35,000 listing)</v>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="5" xml:space="preserve">
+      <c r="A5" t="str">
+        <v>BVA-04</v>
+      </c>
+      <c r="B5" t="str">
+        <v>min_price above the maximum rent returns an empty result set</v>
+      </c>
+      <c r="C5" t="str">
+        <v>8 approved listings; highest rent = ৳35,000</v>
+      </c>
+      <c r="D5" t="str">
+        <v>BVA — just outside the upper boundary; min_price = 35001 yields zero matches</v>
+      </c>
+      <c r="E5" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?min_price=35001
+2. Read the result counter and empty state</v>
+      </c>
+      <c r="F5" t="str">
+        <v>0 rentals found; graceful 'No rentals found' empty state, no server error</v>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6" t="str">
+        <v>BVA-05</v>
+      </c>
+      <c r="B6" t="str">
+        <v>max_price on the lower boundary keeps only the cheapest listing</v>
+      </c>
+      <c r="C6" t="str">
+        <v>8 approved listings; lowest rent = ৳6,000</v>
+      </c>
+      <c r="D6" t="str">
+        <v>BVA — max_price equal to the cheapest rent is inclusive</v>
+      </c>
+      <c r="E6" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?max_price=6000
+2. Read the result counter</v>
+      </c>
+      <c r="F6" t="str">
+        <v>1 rental found (the ৳6,000 listing, rent&lt;=6000 inclusive)</v>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="7" xml:space="preserve">
+      <c r="A7" t="str">
+        <v>BVA-06</v>
+      </c>
+      <c r="B7" t="str">
+        <v>max_price one below the cheapest rent returns an empty result set</v>
+      </c>
+      <c r="C7" t="str">
+        <v>8 approved listings; lowest rent = ৳6,000</v>
+      </c>
+      <c r="D7" t="str">
+        <v>BVA — boundary-1; max_price = 5999 excludes every listing</v>
+      </c>
+      <c r="E7" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?max_price=5999
+2. Read the result counter</v>
+      </c>
+      <c r="F7" t="str">
+        <v>0 rentals found; graceful empty state, no server error</v>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="8" xml:space="preserve">
+      <c r="A8" t="str">
+        <v>BVA-07</v>
+      </c>
+      <c r="B8" t="str">
+        <v>max_price = 0 is treated as 'no upper bound', not 'rent &lt;= 0'</v>
+      </c>
+      <c r="C8" t="str">
+        <v>8 approved listings</v>
+      </c>
+      <c r="D8" t="str">
+        <v>EP/edge — zero is a distinct partition: the unset/no-bound class, not a literal ceiling</v>
+      </c>
+      <c r="E8" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?max_price=0
+2. Read the result counter</v>
+      </c>
+      <c r="F8" t="str">
+        <v>8 rentals found (0 is interpreted as no maximum, the full catalogue is shown)</v>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <v>Low | ep | automated</v>
+      </c>
+    </row>
+    <row r="9" xml:space="preserve">
+      <c r="A9" t="str">
+        <v>EP-01</v>
+      </c>
+      <c r="B9" t="str">
+        <v>bedrooms = Any partition returns the full catalogue</v>
+      </c>
+      <c r="C9" t="str">
+        <v>8 approved listings</v>
+      </c>
+      <c r="D9" t="str">
+        <v>EP — the unfiltered 'Any' partition</v>
+      </c>
+      <c r="E9" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?bedrooms=
+2. Read the result counter</v>
+      </c>
+      <c r="F9" t="str">
+        <v>8 rentals found</v>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
+        <v>Low | ep | automated</v>
+      </c>
+    </row>
+    <row r="10" xml:space="preserve">
+      <c r="A10" t="str">
+        <v>EP-02</v>
+      </c>
+      <c r="B10" t="str">
+        <v>bedrooms = 1+ partition includes every listing</v>
+      </c>
+      <c r="C10" t="str">
+        <v>All listings have at least 1 bedroom</v>
+      </c>
+      <c r="D10" t="str">
+        <v>EP — '1+' class</v>
+      </c>
+      <c r="E10" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?bedrooms=1
+2. Read the result counter</v>
+      </c>
+      <c r="F10" t="str">
+        <v>8 rentals found</v>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10" t="str">
+        <v>Medium | ep | automated</v>
+      </c>
+    </row>
+    <row r="11" xml:space="preserve">
+      <c r="A11" t="str">
+        <v>EP-03</v>
+      </c>
+      <c r="B11" t="str">
+        <v>bedrooms = 2+ partition narrows the result set</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Seed mix of bedroom counts</v>
+      </c>
+      <c r="D11" t="str">
+        <v>EP — '2+' class</v>
+      </c>
+      <c r="E11" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?bedrooms=2
+2. Read the result counter</v>
+      </c>
+      <c r="F11" t="str">
+        <v>5 rentals found (listings with &gt;=2 bedrooms)</v>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11" t="str">
+        <v>Medium | ep | automated</v>
+      </c>
+    </row>
+    <row r="12" xml:space="preserve">
+      <c r="A12" t="str">
+        <v>EP-04</v>
+      </c>
+      <c r="B12" t="str">
+        <v>bedrooms = 3+ partition narrows the result set further</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Seed mix of bedroom counts</v>
+      </c>
+      <c r="D12" t="str">
+        <v>EP — '3+' class (mirrors manual SRCH-04, now automated)</v>
+      </c>
+      <c r="E12" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?bedrooms=3
+2. Read the result counter</v>
+      </c>
+      <c r="F12" t="str">
+        <v>3 rentals found (listings with &gt;=3 bedrooms)</v>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12" t="str">
+        <v>Medium | ep | automated</v>
+      </c>
+    </row>
+    <row r="13" xml:space="preserve">
+      <c r="A13" t="str">
+        <v>EP-05</v>
+      </c>
+      <c r="B13" t="str">
+        <v>bedrooms = 4+ partition keeps only the largest listings</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Seed mix of bedroom counts</v>
+      </c>
+      <c r="D13" t="str">
+        <v>EP — '4+' class (the highest UI option)</v>
+      </c>
+      <c r="E13" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?bedrooms=4
+2. Read the result counter</v>
+      </c>
+      <c r="F13" t="str">
+        <v>1 rental found (listings with &gt;=4 bedrooms)</v>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13" t="str">
+        <v>Medium | ep | automated</v>
+      </c>
+    </row>
+    <row r="14" xml:space="preserve">
+      <c r="A14" t="str">
+        <v>EP-06</v>
+      </c>
+      <c r="B14" t="str">
+        <v>bedrooms = 5 (out-of-range partition) returns an empty result set</v>
+      </c>
+      <c r="C14" t="str">
+        <v>UI offers Any/1+/2+/3+/4+ only; no listing has 5+ bedrooms</v>
+      </c>
+      <c r="D14" t="str">
+        <v>EP/edge — a value beyond the offered partitions is handled gracefully</v>
+      </c>
+      <c r="E14" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?bedrooms=5
+2. Read the result counter and empty state</v>
+      </c>
+      <c r="F14" t="str">
+        <v>0 rentals found; graceful empty state, no server error</v>
+      </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
+      <c r="H14" t="str">
+        <v>Low | edge | automated</v>
+      </c>
+    </row>
+    <row r="15" xml:space="preserve">
+      <c r="A15" t="str">
+        <v>EP-07</v>
+      </c>
+      <c r="B15" t="str">
+        <v>type = family partition returns only Family Flats</v>
+      </c>
+      <c r="C15" t="str">
+        <v>8 approved listings of mixed types; 4 are family</v>
+      </c>
+      <c r="D15" t="str">
+        <v>EP — property-type 'family' class via type[]=family</v>
+      </c>
+      <c r="E15" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?type[]=family
+2. Read the result counter</v>
+      </c>
+      <c r="F15" t="str">
+        <v>4 rentals found (Family Flat listings only)</v>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
+      <c r="H15" t="str">
+        <v>Medium | ep | automated</v>
+      </c>
+    </row>
+    <row r="16" xml:space="preserve">
+      <c r="A16" t="str">
+        <v>EDGE-01</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Inverted price range (min &gt; max) returns an empty set, no crash</v>
+      </c>
+      <c r="C16" t="str">
+        <v>8 approved listings</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Edge — contradictory boundaries; min_price=50000 &amp; max_price=10000</v>
+      </c>
+      <c r="E16" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?min_price=50000&amp;max_price=10000
+2. Read the result counter</v>
+      </c>
+      <c r="F16" t="str">
+        <v>0 rentals found; HTTP 200; graceful empty state (no listing can satisfy both)</v>
+      </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
+      <c r="H16" t="str">
+        <v>Medium | edge | automated</v>
+      </c>
+    </row>
+    <row r="17" xml:space="preserve">
+      <c r="A17" t="str">
+        <v>EDGE-02</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Non-numeric min_price is ignored gracefully</v>
+      </c>
+      <c r="C17" t="str">
+        <v>8 approved listings</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Edge — invalid input class; min_price=abc must not break the page</v>
+      </c>
+      <c r="E17" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?min_price=abc
+2. Read HTTP status and result counter</v>
+      </c>
+      <c r="F17" t="str">
+        <v>HTTP 200; filter ignored; 8 rentals found; no server error or stack trace</v>
+      </c>
+      <c r="G17" t="str">
+        <v/>
+      </c>
+      <c r="H17" t="str">
+        <v>Medium | edge | automated</v>
+      </c>
+    </row>
+    <row r="18" xml:space="preserve">
+      <c r="A18" t="str">
+        <v>EDGE-03</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Negative min_price is ignored gracefully</v>
+      </c>
+      <c r="C18" t="str">
+        <v>8 approved listings</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Edge/BVA — below-zero boundary; min_price=-100 must not break the page</v>
+      </c>
+      <c r="E18" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?min_price=-100
+2. Read HTTP status and result counter</v>
+      </c>
+      <c r="F18" t="str">
+        <v>HTTP 200; negative bound ignored; 8 rentals found; no server error</v>
+      </c>
+      <c r="G18" t="str">
+        <v/>
+      </c>
+      <c r="H18" t="str">
+        <v>Low | edge | automated</v>
+      </c>
+    </row>
+    <row r="19" xml:space="preserve">
+      <c r="A19" t="str">
+        <v>EDGE-04</v>
+      </c>
+      <c r="B19" t="str">
+        <v>No-match search term shows the zero-result empty state</v>
+      </c>
+      <c r="C19" t="str">
+        <v>8 approved listings</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Edge — zero-result query (mirrors manual GUEST-10, now automated)</v>
+      </c>
+      <c r="E19" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?q=Zzzzzz
+2. Read the result counter and empty state</v>
+      </c>
+      <c r="F19" t="str">
+        <v>0 rentals found; 'No rentals found' empty state with a broaden-search hint, no crash</v>
+      </c>
+      <c r="G19" t="str">
+        <v/>
+      </c>
+      <c r="H19" t="str">
+        <v>Medium | edge | automated</v>
+      </c>
+    </row>
+    <row r="20" xml:space="preserve">
+      <c r="A20" t="str">
+        <v>BVA-08</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Password below the 8-character minimum boundary is rejected</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Guest on /register; all other fields valid</v>
+      </c>
+      <c r="D20" t="str">
+        <v>BVA — minimum length boundary-1; a 7-character password must fail validation</v>
+      </c>
+      <c r="E20" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /register
+2. Fill valid name/email/phone/role/terms
+3. Set Password and Confirm to a 7-char value (e.g. 'Pass12!')
+4. Submit</v>
+      </c>
+      <c r="F20" t="str">
+        <v>Inline error 'must be at least 8 characters'; account not created; stays on /register; no HTTP 500</v>
+      </c>
+      <c r="G20" t="str">
+        <v/>
+      </c>
+      <c r="H20" t="str">
+        <v>High | bva | automated</v>
+      </c>
+    </row>
+    <row r="21" xml:space="preserve">
+      <c r="A21" t="str">
+        <v>EP-08</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Phone in the 'too-short numeric' partition is rejected</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Guest on /register; all other fields valid</v>
+      </c>
+      <c r="D21" t="str">
+        <v>EP — invalid phone class; '12345' is not a valid BD number (01XXXXXXXXX / +8801XXXXXXXXX)</v>
+      </c>
+      <c r="E21" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /register
+2. Fill valid name/email/password/role/terms
+3. Set Phone = '12345'
+4. Submit</v>
+      </c>
+      <c r="F21" t="str">
+        <v>Validation rejects the phone; account not created; stays on /register; no HTTP 500</v>
+      </c>
+      <c r="G21" t="str">
+        <v/>
+      </c>
+      <c r="H21" t="str">
+        <v>Medium | ep | automated</v>
+      </c>
+    </row>
+    <row r="22" xml:space="preserve">
+      <c r="A22" t="str">
+        <v>EP-09</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Phone in the 'alphabetic' partition is rejected</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Guest on /register; all other fields valid</v>
+      </c>
+      <c r="D22" t="str">
+        <v>EP — invalid phone class; non-digit input must fail the BD phone rule</v>
+      </c>
+      <c r="E22" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /register
+2. Fill valid name/email/password/role/terms
+3. Set Phone = 'abcdefghijk'
+4. Submit</v>
+      </c>
+      <c r="F22" t="str">
+        <v>Validation rejects the phone; account not created; stays on /register; no HTTP 500</v>
+      </c>
+      <c r="G22" t="str">
+        <v/>
+      </c>
+      <c r="H22" t="str">
+        <v>Medium | ep | automated</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H22"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H81"/>
+  <cols>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="42.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="36.83203125" customWidth="1"/>
+    <col min="5" max="5" width="48.83203125" customWidth="1"/>
+    <col min="6" max="6" width="46.83203125" customWidth="1"/>
+    <col min="7" max="7" width="40.83203125" customWidth="1"/>
+    <col min="8" max="8" width="26.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Title</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Precondition</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Description</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Steps</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Expected Result</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Actual Result</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Comments</v>
+      </c>
+    </row>
+    <row r="2" xml:space="preserve">
+      <c r="A2" t="str">
+        <v>SM-001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>min_price = ৳6000 (inclusive lower boundary)</v>
+      </c>
+      <c r="C2" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Price BVA — /search?min_price=6000</v>
+      </c>
+      <c r="E2" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?min_price=6000
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F2" t="str">
+        <v>8 rentals found</v>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
+      <c r="A3" t="str">
+        <v>SM-002</v>
+      </c>
+      <c r="B3" t="str">
+        <v>min_price = ৳6001 (just above the ৳6000 listing)</v>
+      </c>
+      <c r="C3" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Price BVA — /search?min_price=6001</v>
+      </c>
+      <c r="E3" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?min_price=6001
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F3" t="str">
+        <v>7 rentals found</v>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
+      <c r="A4" t="str">
+        <v>SM-003</v>
+      </c>
+      <c r="B4" t="str">
+        <v>min_price = ৳18000 (inclusive lower boundary)</v>
+      </c>
+      <c r="C4" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Price BVA — /search?min_price=18000</v>
+      </c>
+      <c r="E4" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?min_price=18000
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F4" t="str">
+        <v>7 rentals found</v>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="5" xml:space="preserve">
+      <c r="A5" t="str">
+        <v>SM-004</v>
+      </c>
+      <c r="B5" t="str">
+        <v>min_price = ৳18001 (just above the ৳18000 listing)</v>
+      </c>
+      <c r="C5" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Price BVA — /search?min_price=18001</v>
+      </c>
+      <c r="E5" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?min_price=18001
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F5" t="str">
+        <v>6 rentals found</v>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6" t="str">
+        <v>SM-005</v>
+      </c>
+      <c r="B6" t="str">
+        <v>min_price = ৳20000 (inclusive lower boundary)</v>
+      </c>
+      <c r="C6" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Price BVA — /search?min_price=20000</v>
+      </c>
+      <c r="E6" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?min_price=20000
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F6" t="str">
+        <v>6 rentals found</v>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="7" xml:space="preserve">
+      <c r="A7" t="str">
+        <v>SM-006</v>
+      </c>
+      <c r="B7" t="str">
+        <v>min_price = ৳20001 (just above the ৳20000 listing)</v>
+      </c>
+      <c r="C7" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Price BVA — /search?min_price=20001</v>
+      </c>
+      <c r="E7" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?min_price=20001
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F7" t="str">
+        <v>5 rentals found</v>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="8" xml:space="preserve">
+      <c r="A8" t="str">
+        <v>SM-007</v>
+      </c>
+      <c r="B8" t="str">
+        <v>min_price = ৳22000 (inclusive lower boundary)</v>
+      </c>
+      <c r="C8" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Price BVA — /search?min_price=22000</v>
+      </c>
+      <c r="E8" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?min_price=22000
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F8" t="str">
+        <v>5 rentals found</v>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="9" xml:space="preserve">
+      <c r="A9" t="str">
+        <v>SM-008</v>
+      </c>
+      <c r="B9" t="str">
+        <v>min_price = ৳22001 (just above the ৳22000 listing)</v>
+      </c>
+      <c r="C9" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Price BVA — /search?min_price=22001</v>
+      </c>
+      <c r="E9" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?min_price=22001
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F9" t="str">
+        <v>4 rentals found</v>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="10" xml:space="preserve">
+      <c r="A10" t="str">
+        <v>SM-009</v>
+      </c>
+      <c r="B10" t="str">
+        <v>min_price = ৳25000 (inclusive lower boundary)</v>
+      </c>
+      <c r="C10" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Price BVA — /search?min_price=25000</v>
+      </c>
+      <c r="E10" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?min_price=25000
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F10" t="str">
+        <v>4 rentals found</v>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="11" xml:space="preserve">
+      <c r="A11" t="str">
+        <v>SM-010</v>
+      </c>
+      <c r="B11" t="str">
+        <v>min_price = ৳25001 (just above the ৳25000 listing)</v>
+      </c>
+      <c r="C11" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Price BVA — /search?min_price=25001</v>
+      </c>
+      <c r="E11" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?min_price=25001
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F11" t="str">
+        <v>3 rentals found</v>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="12" xml:space="preserve">
+      <c r="A12" t="str">
+        <v>SM-011</v>
+      </c>
+      <c r="B12" t="str">
+        <v>min_price = ৳28000 (inclusive lower boundary)</v>
+      </c>
+      <c r="C12" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Price BVA — /search?min_price=28000</v>
+      </c>
+      <c r="E12" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?min_price=28000
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F12" t="str">
+        <v>3 rentals found</v>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="13" xml:space="preserve">
+      <c r="A13" t="str">
+        <v>SM-012</v>
+      </c>
+      <c r="B13" t="str">
+        <v>min_price = ৳28001 (just above the ৳28000 listing)</v>
+      </c>
+      <c r="C13" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Price BVA — /search?min_price=28001</v>
+      </c>
+      <c r="E13" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?min_price=28001
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F13" t="str">
+        <v>2 rentals found</v>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="14" xml:space="preserve">
+      <c r="A14" t="str">
+        <v>SM-013</v>
+      </c>
+      <c r="B14" t="str">
+        <v>min_price = ৳32000 (inclusive lower boundary)</v>
+      </c>
+      <c r="C14" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Price BVA — /search?min_price=32000</v>
+      </c>
+      <c r="E14" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?min_price=32000
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F14" t="str">
+        <v>2 rentals found</v>
+      </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
+      <c r="H14" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="15" xml:space="preserve">
+      <c r="A15" t="str">
+        <v>SM-014</v>
+      </c>
+      <c r="B15" t="str">
+        <v>min_price = ৳32001 (just above the ৳32000 listing)</v>
+      </c>
+      <c r="C15" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Price BVA — /search?min_price=32001</v>
+      </c>
+      <c r="E15" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?min_price=32001
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F15" t="str">
+        <v>1 rental found</v>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
+      <c r="H15" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="16" xml:space="preserve">
+      <c r="A16" t="str">
+        <v>SM-015</v>
+      </c>
+      <c r="B16" t="str">
+        <v>min_price = ৳35000 (inclusive lower boundary)</v>
+      </c>
+      <c r="C16" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Price BVA — /search?min_price=35000</v>
+      </c>
+      <c r="E16" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?min_price=35000
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F16" t="str">
+        <v>1 rental found</v>
+      </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
+      <c r="H16" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="17" xml:space="preserve">
+      <c r="A17" t="str">
+        <v>SM-016</v>
+      </c>
+      <c r="B17" t="str">
+        <v>min_price = ৳35001 (just above the ৳35000 listing)</v>
+      </c>
+      <c r="C17" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Price BVA — /search?min_price=35001</v>
+      </c>
+      <c r="E17" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?min_price=35001
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F17" t="str">
+        <v>0 rentals found</v>
+      </c>
+      <c r="G17" t="str">
+        <v/>
+      </c>
+      <c r="H17" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="18" xml:space="preserve">
+      <c r="A18" t="str">
+        <v>SM-017</v>
+      </c>
+      <c r="B18" t="str">
+        <v>max_price = ৳6000 (inclusive upper boundary)</v>
+      </c>
+      <c r="C18" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Price BVA — /search?max_price=6000</v>
+      </c>
+      <c r="E18" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?max_price=6000
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F18" t="str">
+        <v>1 rental found</v>
+      </c>
+      <c r="G18" t="str">
+        <v/>
+      </c>
+      <c r="H18" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="19" xml:space="preserve">
+      <c r="A19" t="str">
+        <v>SM-018</v>
+      </c>
+      <c r="B19" t="str">
+        <v>max_price = ৳5999 (just below the ৳6000 listing)</v>
+      </c>
+      <c r="C19" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Price BVA — /search?max_price=5999</v>
+      </c>
+      <c r="E19" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?max_price=5999
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F19" t="str">
+        <v>0 rentals found</v>
+      </c>
+      <c r="G19" t="str">
+        <v/>
+      </c>
+      <c r="H19" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="20" xml:space="preserve">
+      <c r="A20" t="str">
+        <v>SM-019</v>
+      </c>
+      <c r="B20" t="str">
+        <v>max_price = ৳18000 (inclusive upper boundary)</v>
+      </c>
+      <c r="C20" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Price BVA — /search?max_price=18000</v>
+      </c>
+      <c r="E20" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?max_price=18000
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F20" t="str">
+        <v>2 rentals found</v>
+      </c>
+      <c r="G20" t="str">
+        <v/>
+      </c>
+      <c r="H20" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="21" xml:space="preserve">
+      <c r="A21" t="str">
+        <v>SM-020</v>
+      </c>
+      <c r="B21" t="str">
+        <v>max_price = ৳17999 (just below the ৳18000 listing)</v>
+      </c>
+      <c r="C21" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Price BVA — /search?max_price=17999</v>
+      </c>
+      <c r="E21" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?max_price=17999
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F21" t="str">
+        <v>1 rental found</v>
+      </c>
+      <c r="G21" t="str">
+        <v/>
+      </c>
+      <c r="H21" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="22" xml:space="preserve">
+      <c r="A22" t="str">
+        <v>SM-021</v>
+      </c>
+      <c r="B22" t="str">
+        <v>max_price = ৳20000 (inclusive upper boundary)</v>
+      </c>
+      <c r="C22" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Price BVA — /search?max_price=20000</v>
+      </c>
+      <c r="E22" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?max_price=20000
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F22" t="str">
+        <v>3 rentals found</v>
+      </c>
+      <c r="G22" t="str">
+        <v/>
+      </c>
+      <c r="H22" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="23" xml:space="preserve">
+      <c r="A23" t="str">
+        <v>SM-022</v>
+      </c>
+      <c r="B23" t="str">
+        <v>max_price = ৳19999 (just below the ৳20000 listing)</v>
+      </c>
+      <c r="C23" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Price BVA — /search?max_price=19999</v>
+      </c>
+      <c r="E23" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?max_price=19999
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F23" t="str">
+        <v>2 rentals found</v>
+      </c>
+      <c r="G23" t="str">
+        <v/>
+      </c>
+      <c r="H23" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="24" xml:space="preserve">
+      <c r="A24" t="str">
+        <v>SM-023</v>
+      </c>
+      <c r="B24" t="str">
+        <v>max_price = ৳22000 (inclusive upper boundary)</v>
+      </c>
+      <c r="C24" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Price BVA — /search?max_price=22000</v>
+      </c>
+      <c r="E24" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?max_price=22000
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F24" t="str">
+        <v>4 rentals found</v>
+      </c>
+      <c r="G24" t="str">
+        <v/>
+      </c>
+      <c r="H24" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="25" xml:space="preserve">
+      <c r="A25" t="str">
+        <v>SM-024</v>
+      </c>
+      <c r="B25" t="str">
+        <v>max_price = ৳21999 (just below the ৳22000 listing)</v>
+      </c>
+      <c r="C25" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Price BVA — /search?max_price=21999</v>
+      </c>
+      <c r="E25" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?max_price=21999
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F25" t="str">
+        <v>3 rentals found</v>
+      </c>
+      <c r="G25" t="str">
+        <v/>
+      </c>
+      <c r="H25" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="26" xml:space="preserve">
+      <c r="A26" t="str">
+        <v>SM-025</v>
+      </c>
+      <c r="B26" t="str">
+        <v>max_price = ৳25000 (inclusive upper boundary)</v>
+      </c>
+      <c r="C26" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Price BVA — /search?max_price=25000</v>
+      </c>
+      <c r="E26" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?max_price=25000
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F26" t="str">
+        <v>5 rentals found</v>
+      </c>
+      <c r="G26" t="str">
+        <v/>
+      </c>
+      <c r="H26" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="27" xml:space="preserve">
+      <c r="A27" t="str">
+        <v>SM-026</v>
+      </c>
+      <c r="B27" t="str">
+        <v>max_price = ৳24999 (just below the ৳25000 listing)</v>
+      </c>
+      <c r="C27" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Price BVA — /search?max_price=24999</v>
+      </c>
+      <c r="E27" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?max_price=24999
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F27" t="str">
+        <v>4 rentals found</v>
+      </c>
+      <c r="G27" t="str">
+        <v/>
+      </c>
+      <c r="H27" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="28" xml:space="preserve">
+      <c r="A28" t="str">
+        <v>SM-027</v>
+      </c>
+      <c r="B28" t="str">
+        <v>max_price = ৳28000 (inclusive upper boundary)</v>
+      </c>
+      <c r="C28" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Price BVA — /search?max_price=28000</v>
+      </c>
+      <c r="E28" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?max_price=28000
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F28" t="str">
+        <v>6 rentals found</v>
+      </c>
+      <c r="G28" t="str">
+        <v/>
+      </c>
+      <c r="H28" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="29" xml:space="preserve">
+      <c r="A29" t="str">
+        <v>SM-028</v>
+      </c>
+      <c r="B29" t="str">
+        <v>max_price = ৳27999 (just below the ৳28000 listing)</v>
+      </c>
+      <c r="C29" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Price BVA — /search?max_price=27999</v>
+      </c>
+      <c r="E29" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?max_price=27999
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F29" t="str">
+        <v>5 rentals found</v>
+      </c>
+      <c r="G29" t="str">
+        <v/>
+      </c>
+      <c r="H29" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="30" xml:space="preserve">
+      <c r="A30" t="str">
+        <v>SM-029</v>
+      </c>
+      <c r="B30" t="str">
+        <v>max_price = ৳32000 (inclusive upper boundary)</v>
+      </c>
+      <c r="C30" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Price BVA — /search?max_price=32000</v>
+      </c>
+      <c r="E30" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?max_price=32000
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F30" t="str">
+        <v>7 rentals found</v>
+      </c>
+      <c r="G30" t="str">
+        <v/>
+      </c>
+      <c r="H30" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="31" xml:space="preserve">
+      <c r="A31" t="str">
+        <v>SM-030</v>
+      </c>
+      <c r="B31" t="str">
+        <v>max_price = ৳31999 (just below the ৳32000 listing)</v>
+      </c>
+      <c r="C31" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Price BVA — /search?max_price=31999</v>
+      </c>
+      <c r="E31" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?max_price=31999
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F31" t="str">
+        <v>6 rentals found</v>
+      </c>
+      <c r="G31" t="str">
+        <v/>
+      </c>
+      <c r="H31" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="32" xml:space="preserve">
+      <c r="A32" t="str">
+        <v>SM-031</v>
+      </c>
+      <c r="B32" t="str">
+        <v>max_price = ৳35000 (inclusive upper boundary)</v>
+      </c>
+      <c r="C32" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Price BVA — /search?max_price=35000</v>
+      </c>
+      <c r="E32" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?max_price=35000
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F32" t="str">
+        <v>8 rentals found</v>
+      </c>
+      <c r="G32" t="str">
+        <v/>
+      </c>
+      <c r="H32" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="33" xml:space="preserve">
+      <c r="A33" t="str">
+        <v>SM-032</v>
+      </c>
+      <c r="B33" t="str">
+        <v>max_price = ৳34999 (just below the ৳35000 listing)</v>
+      </c>
+      <c r="C33" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Price BVA — /search?max_price=34999</v>
+      </c>
+      <c r="E33" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?max_price=34999
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F33" t="str">
+        <v>7 rentals found</v>
+      </c>
+      <c r="G33" t="str">
+        <v/>
+      </c>
+      <c r="H33" t="str">
+        <v>Medium | bva | automated</v>
+      </c>
+    </row>
+    <row r="34" xml:space="preserve">
+      <c r="A34" t="str">
+        <v>SM-033</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Property type = 'family'</v>
+      </c>
+      <c r="C34" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Type EP — /search?type[]=family</v>
+      </c>
+      <c r="E34" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?type[]=family
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F34" t="str">
+        <v>4 rentals found</v>
+      </c>
+      <c r="G34" t="str">
+        <v/>
+      </c>
+      <c r="H34" t="str">
+        <v>Medium | ep | automated</v>
+      </c>
+    </row>
+    <row r="35" xml:space="preserve">
+      <c r="A35" t="str">
+        <v>SM-034</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Property type = 'bachelor'</v>
+      </c>
+      <c r="C35" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Type EP — /search?type[]=bachelor</v>
+      </c>
+      <c r="E35" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?type[]=bachelor
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F35" t="str">
+        <v>1 rental found</v>
+      </c>
+      <c r="G35" t="str">
+        <v/>
+      </c>
+      <c r="H35" t="str">
+        <v>Medium | ep | automated</v>
+      </c>
+    </row>
+    <row r="36" xml:space="preserve">
+      <c r="A36" t="str">
+        <v>SM-035</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Property type = 'sublet'</v>
+      </c>
+      <c r="C36" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Type EP — /search?type[]=sublet</v>
+      </c>
+      <c r="E36" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?type[]=sublet
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F36" t="str">
+        <v>2 rentals found</v>
+      </c>
+      <c r="G36" t="str">
+        <v/>
+      </c>
+      <c r="H36" t="str">
+        <v>Medium | ep | automated</v>
+      </c>
+    </row>
+    <row r="37" xml:space="preserve">
+      <c r="A37" t="str">
+        <v>SM-036</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Property type = 'shared'</v>
+      </c>
+      <c r="C37" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Type EP — /search?type[]=shared</v>
+      </c>
+      <c r="E37" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?type[]=shared
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F37" t="str">
+        <v>1 rental found</v>
+      </c>
+      <c r="G37" t="str">
+        <v/>
+      </c>
+      <c r="H37" t="str">
+        <v>Medium | ep | automated</v>
+      </c>
+    </row>
+    <row r="38" xml:space="preserve">
+      <c r="A38" t="str">
+        <v>SM-037</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Property type = 'hostel'</v>
+      </c>
+      <c r="C38" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Type EP — /search?type[]=hostel</v>
+      </c>
+      <c r="E38" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?type[]=hostel
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F38" t="str">
+        <v>0 rentals found</v>
+      </c>
+      <c r="G38" t="str">
+        <v/>
+      </c>
+      <c r="H38" t="str">
+        <v>Medium | ep | automated</v>
+      </c>
+    </row>
+    <row r="39" xml:space="preserve">
+      <c r="A39" t="str">
+        <v>SM-038</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Property type = 'garage'</v>
+      </c>
+      <c r="C39" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Type EP — /search?type[]=garage</v>
+      </c>
+      <c r="E39" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?type[]=garage
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F39" t="str">
+        <v>0 rentals found</v>
+      </c>
+      <c r="G39" t="str">
+        <v/>
+      </c>
+      <c r="H39" t="str">
+        <v>Medium | ep | automated</v>
+      </c>
+    </row>
+    <row r="40" xml:space="preserve">
+      <c r="A40" t="str">
+        <v>SM-039</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Suitable for = 'family'</v>
+      </c>
+      <c r="C40" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D40" t="str">
+        <v>ForWhom EP — /search?for_whom=family</v>
+      </c>
+      <c r="E40" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?for_whom=family
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F40" t="str">
+        <v>6 rentals found</v>
+      </c>
+      <c r="G40" t="str">
+        <v/>
+      </c>
+      <c r="H40" t="str">
+        <v>Medium | ep | automated</v>
+      </c>
+    </row>
+    <row r="41" xml:space="preserve">
+      <c r="A41" t="str">
+        <v>SM-040</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Suitable for = 'bachelor'</v>
+      </c>
+      <c r="C41" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D41" t="str">
+        <v>ForWhom EP — /search?for_whom=bachelor</v>
+      </c>
+      <c r="E41" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?for_whom=bachelor
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F41" t="str">
+        <v>5 rentals found</v>
+      </c>
+      <c r="G41" t="str">
+        <v/>
+      </c>
+      <c r="H41" t="str">
+        <v>Medium | ep | automated</v>
+      </c>
+    </row>
+    <row r="42" xml:space="preserve">
+      <c r="A42" t="str">
+        <v>SM-041</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Furnishing = 'unfurnished'</v>
+      </c>
+      <c r="C42" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Furnishing EP — /search?furnishing[]=unfurnished</v>
+      </c>
+      <c r="E42" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?furnishing[]=unfurnished
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F42" t="str">
+        <v>3 rentals found</v>
+      </c>
+      <c r="G42" t="str">
+        <v/>
+      </c>
+      <c r="H42" t="str">
+        <v>Medium | ep | automated</v>
+      </c>
+    </row>
+    <row r="43" xml:space="preserve">
+      <c r="A43" t="str">
+        <v>SM-042</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Furnishing = 'semi_furnished'</v>
+      </c>
+      <c r="C43" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Furnishing EP — /search?furnishing[]=semi_furnished</v>
+      </c>
+      <c r="E43" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?furnishing[]=semi_furnished
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F43" t="str">
+        <v>3 rentals found</v>
+      </c>
+      <c r="G43" t="str">
+        <v/>
+      </c>
+      <c r="H43" t="str">
+        <v>Medium | ep | automated</v>
+      </c>
+    </row>
+    <row r="44" xml:space="preserve">
+      <c r="A44" t="str">
+        <v>SM-043</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Furnishing = 'fully_furnished'</v>
+      </c>
+      <c r="C44" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Furnishing EP — /search?furnishing[]=fully_furnished</v>
+      </c>
+      <c r="E44" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?furnishing[]=fully_furnished
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F44" t="str">
+        <v>2 rentals found</v>
+      </c>
+      <c r="G44" t="str">
+        <v/>
+      </c>
+      <c r="H44" t="str">
+        <v>Medium | ep | automated</v>
+      </c>
+    </row>
+    <row r="45" xml:space="preserve">
+      <c r="A45" t="str">
+        <v>SM-044</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Amenity id=1 filter</v>
+      </c>
+      <c r="C45" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Amenity EP — /search?amenities[]=1</v>
+      </c>
+      <c r="E45" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?amenities[]=1
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F45" t="str">
+        <v>3 rentals found</v>
+      </c>
+      <c r="G45" t="str">
+        <v/>
+      </c>
+      <c r="H45" t="str">
+        <v>Low | ep | automated</v>
+      </c>
+    </row>
+    <row r="46" xml:space="preserve">
+      <c r="A46" t="str">
+        <v>SM-045</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Amenity id=2 filter</v>
+      </c>
+      <c r="C46" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D46" t="str">
+        <v>Amenity EP — /search?amenities[]=2</v>
+      </c>
+      <c r="E46" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?amenities[]=2
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F46" t="str">
+        <v>1 rental found</v>
+      </c>
+      <c r="G46" t="str">
+        <v/>
+      </c>
+      <c r="H46" t="str">
+        <v>Low | ep | automated</v>
+      </c>
+    </row>
+    <row r="47" xml:space="preserve">
+      <c r="A47" t="str">
+        <v>SM-046</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Amenity id=3 filter</v>
+      </c>
+      <c r="C47" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D47" t="str">
+        <v>Amenity EP — /search?amenities[]=3</v>
+      </c>
+      <c r="E47" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?amenities[]=3
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F47" t="str">
+        <v>1 rental found</v>
+      </c>
+      <c r="G47" t="str">
+        <v/>
+      </c>
+      <c r="H47" t="str">
+        <v>Low | ep | automated</v>
+      </c>
+    </row>
+    <row r="48" xml:space="preserve">
+      <c r="A48" t="str">
+        <v>SM-047</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Amenity id=4 filter</v>
+      </c>
+      <c r="C48" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Amenity EP — /search?amenities[]=4</v>
+      </c>
+      <c r="E48" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?amenities[]=4
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F48" t="str">
+        <v>3 rentals found</v>
+      </c>
+      <c r="G48" t="str">
+        <v/>
+      </c>
+      <c r="H48" t="str">
+        <v>Low | ep | automated</v>
+      </c>
+    </row>
+    <row r="49" xml:space="preserve">
+      <c r="A49" t="str">
+        <v>SM-048</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Amenity id=5 filter</v>
+      </c>
+      <c r="C49" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Amenity EP — /search?amenities[]=5</v>
+      </c>
+      <c r="E49" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?amenities[]=5
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F49" t="str">
+        <v>1 rental found</v>
+      </c>
+      <c r="G49" t="str">
+        <v/>
+      </c>
+      <c r="H49" t="str">
+        <v>Low | ep | automated</v>
+      </c>
+    </row>
+    <row r="50" xml:space="preserve">
+      <c r="A50" t="str">
+        <v>SM-049</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Amenity id=6 filter</v>
+      </c>
+      <c r="C50" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D50" t="str">
+        <v>Amenity EP — /search?amenities[]=6</v>
+      </c>
+      <c r="E50" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?amenities[]=6
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F50" t="str">
+        <v>1 rental found</v>
+      </c>
+      <c r="G50" t="str">
+        <v/>
+      </c>
+      <c r="H50" t="str">
+        <v>Low | ep | automated</v>
+      </c>
+    </row>
+    <row r="51" xml:space="preserve">
+      <c r="A51" t="str">
+        <v>SM-050</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Amenity id=7 filter</v>
+      </c>
+      <c r="C51" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D51" t="str">
+        <v>Amenity EP — /search?amenities[]=7</v>
+      </c>
+      <c r="E51" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?amenities[]=7
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F51" t="str">
+        <v>1 rental found</v>
+      </c>
+      <c r="G51" t="str">
+        <v/>
+      </c>
+      <c r="H51" t="str">
+        <v>Low | ep | automated</v>
+      </c>
+    </row>
+    <row r="52" xml:space="preserve">
+      <c r="A52" t="str">
+        <v>SM-051</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Amenity id=8 filter</v>
+      </c>
+      <c r="C52" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D52" t="str">
+        <v>Amenity EP — /search?amenities[]=8</v>
+      </c>
+      <c r="E52" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?amenities[]=8
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F52" t="str">
+        <v>3 rentals found</v>
+      </c>
+      <c r="G52" t="str">
+        <v/>
+      </c>
+      <c r="H52" t="str">
+        <v>Low | ep | automated</v>
+      </c>
+    </row>
+    <row r="53" xml:space="preserve">
+      <c r="A53" t="str">
+        <v>SM-052</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Amenity id=9 filter</v>
+      </c>
+      <c r="C53" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D53" t="str">
+        <v>Amenity EP — /search?amenities[]=9</v>
+      </c>
+      <c r="E53" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?amenities[]=9
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F53" t="str">
+        <v>0 rentals found</v>
+      </c>
+      <c r="G53" t="str">
+        <v/>
+      </c>
+      <c r="H53" t="str">
+        <v>Low | ep | automated</v>
+      </c>
+    </row>
+    <row r="54" xml:space="preserve">
+      <c r="A54" t="str">
+        <v>SM-053</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Amenity id=10 filter</v>
+      </c>
+      <c r="C54" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D54" t="str">
+        <v>Amenity EP — /search?amenities[]=10</v>
+      </c>
+      <c r="E54" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?amenities[]=10
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F54" t="str">
+        <v>3 rentals found</v>
+      </c>
+      <c r="G54" t="str">
+        <v/>
+      </c>
+      <c r="H54" t="str">
+        <v>Low | ep | automated</v>
+      </c>
+    </row>
+    <row r="55" xml:space="preserve">
+      <c r="A55" t="str">
+        <v>SM-054</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Amenity id=11 filter</v>
+      </c>
+      <c r="C55" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D55" t="str">
+        <v>Amenity EP — /search?amenities[]=11</v>
+      </c>
+      <c r="E55" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?amenities[]=11
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F55" t="str">
+        <v>1 rental found</v>
+      </c>
+      <c r="G55" t="str">
+        <v/>
+      </c>
+      <c r="H55" t="str">
+        <v>Low | ep | automated</v>
+      </c>
+    </row>
+    <row r="56" xml:space="preserve">
+      <c r="A56" t="str">
+        <v>SM-055</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Amenity id=12 filter</v>
+      </c>
+      <c r="C56" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D56" t="str">
+        <v>Amenity EP — /search?amenities[]=12</v>
+      </c>
+      <c r="E56" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?amenities[]=12
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F56" t="str">
+        <v>0 rentals found</v>
+      </c>
+      <c r="G56" t="str">
+        <v/>
+      </c>
+      <c r="H56" t="str">
+        <v>Low | ep | automated</v>
+      </c>
+    </row>
+    <row r="57" xml:space="preserve">
+      <c r="A57" t="str">
+        <v>SM-056</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Amenity id=13 filter</v>
+      </c>
+      <c r="C57" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D57" t="str">
+        <v>Amenity EP — /search?amenities[]=13</v>
+      </c>
+      <c r="E57" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?amenities[]=13
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F57" t="str">
+        <v>0 rentals found</v>
+      </c>
+      <c r="G57" t="str">
+        <v/>
+      </c>
+      <c r="H57" t="str">
+        <v>Low | ep | automated</v>
+      </c>
+    </row>
+    <row r="58" xml:space="preserve">
+      <c r="A58" t="str">
+        <v>SM-057</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Amenity id=14 filter</v>
+      </c>
+      <c r="C58" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D58" t="str">
+        <v>Amenity EP — /search?amenities[]=14</v>
+      </c>
+      <c r="E58" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?amenities[]=14
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F58" t="str">
+        <v>2 rentals found</v>
+      </c>
+      <c r="G58" t="str">
+        <v/>
+      </c>
+      <c r="H58" t="str">
+        <v>Low | ep | automated</v>
+      </c>
+    </row>
+    <row r="59" xml:space="preserve">
+      <c r="A59" t="str">
+        <v>SM-058</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Amenity id=15 filter</v>
+      </c>
+      <c r="C59" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D59" t="str">
+        <v>Amenity EP — /search?amenities[]=15</v>
+      </c>
+      <c r="E59" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?amenities[]=15
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F59" t="str">
+        <v>0 rentals found</v>
+      </c>
+      <c r="G59" t="str">
+        <v/>
+      </c>
+      <c r="H59" t="str">
+        <v>Low | ep | automated</v>
+      </c>
+    </row>
+    <row r="60" xml:space="preserve">
+      <c r="A60" t="str">
+        <v>SM-059</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Amenity id=16 filter</v>
+      </c>
+      <c r="C60" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D60" t="str">
+        <v>Amenity EP — /search?amenities[]=16</v>
+      </c>
+      <c r="E60" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?amenities[]=16
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F60" t="str">
+        <v>1 rental found</v>
+      </c>
+      <c r="G60" t="str">
+        <v/>
+      </c>
+      <c r="H60" t="str">
+        <v>Low | ep | automated</v>
+      </c>
+    </row>
+    <row r="61" xml:space="preserve">
+      <c r="A61" t="str">
+        <v>SM-060</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Amenity id=17 filter</v>
+      </c>
+      <c r="C61" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D61" t="str">
+        <v>Amenity EP — /search?amenities[]=17</v>
+      </c>
+      <c r="E61" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?amenities[]=17
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F61" t="str">
+        <v>1 rental found</v>
+      </c>
+      <c r="G61" t="str">
+        <v/>
+      </c>
+      <c r="H61" t="str">
+        <v>Low | ep | automated</v>
+      </c>
+    </row>
+    <row r="62" xml:space="preserve">
+      <c r="A62" t="str">
+        <v>SM-061</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Amenity id=18 filter</v>
+      </c>
+      <c r="C62" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D62" t="str">
+        <v>Amenity EP — /search?amenities[]=18</v>
+      </c>
+      <c r="E62" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?amenities[]=18
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F62" t="str">
+        <v>1 rental found</v>
+      </c>
+      <c r="G62" t="str">
+        <v/>
+      </c>
+      <c r="H62" t="str">
+        <v>Low | ep | automated</v>
+      </c>
+    </row>
+    <row r="63" xml:space="preserve">
+      <c r="A63" t="str">
+        <v>SM-062</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Amenity id=19 filter</v>
+      </c>
+      <c r="C63" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D63" t="str">
+        <v>Amenity EP — /search?amenities[]=19</v>
+      </c>
+      <c r="E63" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?amenities[]=19
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F63" t="str">
+        <v>1 rental found</v>
+      </c>
+      <c r="G63" t="str">
+        <v/>
+      </c>
+      <c r="H63" t="str">
+        <v>Low | ep | automated</v>
+      </c>
+    </row>
+    <row r="64" xml:space="preserve">
+      <c r="A64" t="str">
+        <v>SM-063</v>
+      </c>
+      <c r="B64" t="str">
+        <v>Amenity id=20 filter</v>
+      </c>
+      <c r="C64" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D64" t="str">
+        <v>Amenity EP — /search?amenities[]=20</v>
+      </c>
+      <c r="E64" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?amenities[]=20
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F64" t="str">
+        <v>1 rental found</v>
+      </c>
+      <c r="G64" t="str">
+        <v/>
+      </c>
+      <c r="H64" t="str">
+        <v>Low | ep | automated</v>
+      </c>
+    </row>
+    <row r="65" xml:space="preserve">
+      <c r="A65" t="str">
+        <v>SM-064</v>
+      </c>
+      <c r="B65" t="str">
+        <v>Amenity id=21 filter</v>
+      </c>
+      <c r="C65" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D65" t="str">
+        <v>Amenity EP — /search?amenities[]=21</v>
+      </c>
+      <c r="E65" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?amenities[]=21
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F65" t="str">
+        <v>0 rentals found</v>
+      </c>
+      <c r="G65" t="str">
+        <v/>
+      </c>
+      <c r="H65" t="str">
+        <v>Low | ep | automated</v>
+      </c>
+    </row>
+    <row r="66" xml:space="preserve">
+      <c r="A66" t="str">
+        <v>SM-065</v>
+      </c>
+      <c r="B66" t="str">
+        <v>Amenity id=22 filter</v>
+      </c>
+      <c r="C66" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D66" t="str">
+        <v>Amenity EP — /search?amenities[]=22</v>
+      </c>
+      <c r="E66" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?amenities[]=22
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F66" t="str">
+        <v>2 rentals found</v>
+      </c>
+      <c r="G66" t="str">
+        <v/>
+      </c>
+      <c r="H66" t="str">
+        <v>Low | ep | automated</v>
+      </c>
+    </row>
+    <row r="67" xml:space="preserve">
+      <c r="A67" t="str">
+        <v>SM-066</v>
+      </c>
+      <c r="B67" t="str">
+        <v>Amenity id=23 filter</v>
+      </c>
+      <c r="C67" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D67" t="str">
+        <v>Amenity EP — /search?amenities[]=23</v>
+      </c>
+      <c r="E67" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?amenities[]=23
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F67" t="str">
+        <v>1 rental found</v>
+      </c>
+      <c r="G67" t="str">
+        <v/>
+      </c>
+      <c r="H67" t="str">
+        <v>Low | ep | automated</v>
+      </c>
+    </row>
+    <row r="68" xml:space="preserve">
+      <c r="A68" t="str">
+        <v>SM-067</v>
+      </c>
+      <c r="B68" t="str">
+        <v>Amenity id=24 filter</v>
+      </c>
+      <c r="C68" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D68" t="str">
+        <v>Amenity EP — /search?amenities[]=24</v>
+      </c>
+      <c r="E68" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?amenities[]=24
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F68" t="str">
+        <v>1 rental found</v>
+      </c>
+      <c r="G68" t="str">
+        <v/>
+      </c>
+      <c r="H68" t="str">
+        <v>Low | ep | automated</v>
+      </c>
+    </row>
+    <row r="69" xml:space="preserve">
+      <c r="A69" t="str">
+        <v>SM-068</v>
+      </c>
+      <c r="B69" t="str">
+        <v>Amenity id=25 filter</v>
+      </c>
+      <c r="C69" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D69" t="str">
+        <v>Amenity EP — /search?amenities[]=25</v>
+      </c>
+      <c r="E69" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?amenities[]=25
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F69" t="str">
+        <v>2 rentals found</v>
+      </c>
+      <c r="G69" t="str">
+        <v/>
+      </c>
+      <c r="H69" t="str">
+        <v>Low | ep | automated</v>
+      </c>
+    </row>
+    <row r="70" xml:space="preserve">
+      <c r="A70" t="str">
+        <v>SM-069</v>
+      </c>
+      <c r="B70" t="str">
+        <v>Amenity id=26 filter</v>
+      </c>
+      <c r="C70" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D70" t="str">
+        <v>Amenity EP — /search?amenities[]=26</v>
+      </c>
+      <c r="E70" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?amenities[]=26
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F70" t="str">
+        <v>0 rentals found</v>
+      </c>
+      <c r="G70" t="str">
+        <v/>
+      </c>
+      <c r="H70" t="str">
+        <v>Low | ep | automated</v>
+      </c>
+    </row>
+    <row r="71" xml:space="preserve">
+      <c r="A71" t="str">
+        <v>SM-070</v>
+      </c>
+      <c r="B71" t="str">
+        <v>Amenity id=27 filter</v>
+      </c>
+      <c r="C71" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D71" t="str">
+        <v>Amenity EP — /search?amenities[]=27</v>
+      </c>
+      <c r="E71" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?amenities[]=27
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F71" t="str">
+        <v>1 rental found</v>
+      </c>
+      <c r="G71" t="str">
+        <v/>
+      </c>
+      <c r="H71" t="str">
+        <v>Low | ep | automated</v>
+      </c>
+    </row>
+    <row r="72" xml:space="preserve">
+      <c r="A72" t="str">
+        <v>SM-071</v>
+      </c>
+      <c r="B72" t="str">
+        <v>family flats with &gt;=2 bedrooms</v>
+      </c>
+      <c r="C72" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D72" t="str">
+        <v>Combined EP — /search?type[]=family&amp;bedrooms=2</v>
+      </c>
+      <c r="E72" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?type[]=family&amp;bedrooms=2
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F72" t="str">
+        <v>4 rentals found</v>
+      </c>
+      <c r="G72" t="str">
+        <v/>
+      </c>
+      <c r="H72" t="str">
+        <v>Medium | ep | automated</v>
+      </c>
+    </row>
+    <row r="73" xml:space="preserve">
+      <c r="A73" t="str">
+        <v>SM-072</v>
+      </c>
+      <c r="B73" t="str">
+        <v>family flats from ৳20,000</v>
+      </c>
+      <c r="C73" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D73" t="str">
+        <v>Combined EP — /search?type[]=family&amp;min_price=20000</v>
+      </c>
+      <c r="E73" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?type[]=family&amp;min_price=20000
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F73" t="str">
+        <v>4 rentals found</v>
+      </c>
+      <c r="G73" t="str">
+        <v/>
+      </c>
+      <c r="H73" t="str">
+        <v>Medium | ep | automated</v>
+      </c>
+    </row>
+    <row r="74" xml:space="preserve">
+      <c r="A74" t="str">
+        <v>SM-073</v>
+      </c>
+      <c r="B74" t="str">
+        <v>&gt;=3 bedrooms, fully furnished</v>
+      </c>
+      <c r="C74" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D74" t="str">
+        <v>Combined EP — /search?bedrooms=3&amp;furnishing[]=fully_furnished</v>
+      </c>
+      <c r="E74" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?bedrooms=3&amp;furnishing[]=fully_furnished
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F74" t="str">
+        <v>0 rentals found</v>
+      </c>
+      <c r="G74" t="str">
+        <v/>
+      </c>
+      <c r="H74" t="str">
+        <v>Medium | ep | automated</v>
+      </c>
+    </row>
+    <row r="75" xml:space="preserve">
+      <c r="A75" t="str">
+        <v>SM-074</v>
+      </c>
+      <c r="B75" t="str">
+        <v>bachelor up to ৳20,000</v>
+      </c>
+      <c r="C75" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D75" t="str">
+        <v>Combined EP — /search?type[]=bachelor&amp;max_price=20000</v>
+      </c>
+      <c r="E75" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?type[]=bachelor&amp;max_price=20000
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F75" t="str">
+        <v>1 rental found</v>
+      </c>
+      <c r="G75" t="str">
+        <v/>
+      </c>
+      <c r="H75" t="str">
+        <v>Medium | ep | automated</v>
+      </c>
+    </row>
+    <row r="76" xml:space="preserve">
+      <c r="A76" t="str">
+        <v>SM-075</v>
+      </c>
+      <c r="B76" t="str">
+        <v>for family, &gt;=2 bedrooms</v>
+      </c>
+      <c r="C76" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D76" t="str">
+        <v>Combined EP — /search?for_whom=family&amp;bedrooms=2</v>
+      </c>
+      <c r="E76" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?for_whom=family&amp;bedrooms=2
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F76" t="str">
+        <v>4 rentals found</v>
+      </c>
+      <c r="G76" t="str">
+        <v/>
+      </c>
+      <c r="H76" t="str">
+        <v>Medium | ep | automated</v>
+      </c>
+    </row>
+    <row r="77" xml:space="preserve">
+      <c r="A77" t="str">
+        <v>SM-076</v>
+      </c>
+      <c r="B77" t="str">
+        <v>rent between ৳20,000 and ৳30,000</v>
+      </c>
+      <c r="C77" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D77" t="str">
+        <v>Combined EP — /search?min_price=20000&amp;max_price=30000</v>
+      </c>
+      <c r="E77" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?min_price=20000&amp;max_price=30000
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F77" t="str">
+        <v>4 rentals found</v>
+      </c>
+      <c r="G77" t="str">
+        <v/>
+      </c>
+      <c r="H77" t="str">
+        <v>Medium | ep | automated</v>
+      </c>
+    </row>
+    <row r="78" xml:space="preserve">
+      <c r="A78" t="str">
+        <v>SM-077</v>
+      </c>
+      <c r="B78" t="str">
+        <v>family OR bachelor (multi-type)</v>
+      </c>
+      <c r="C78" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D78" t="str">
+        <v>Combined EP — /search?type[]=family&amp;type[]=bachelor</v>
+      </c>
+      <c r="E78" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?type[]=family&amp;type[]=bachelor
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F78" t="str">
+        <v>5 rentals found</v>
+      </c>
+      <c r="G78" t="str">
+        <v/>
+      </c>
+      <c r="H78" t="str">
+        <v>Medium | ep | automated</v>
+      </c>
+    </row>
+    <row r="79" xml:space="preserve">
+      <c r="A79" t="str">
+        <v>SM-078</v>
+      </c>
+      <c r="B79" t="str">
+        <v>fully furnished for family</v>
+      </c>
+      <c r="C79" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D79" t="str">
+        <v>Combined EP — /search?furnishing[]=fully_furnished&amp;for_whom=family</v>
+      </c>
+      <c r="E79" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?furnishing[]=fully_furnished&amp;for_whom=family
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F79" t="str">
+        <v>2 rentals found</v>
+      </c>
+      <c r="G79" t="str">
+        <v/>
+      </c>
+      <c r="H79" t="str">
+        <v>Medium | ep | automated</v>
+      </c>
+    </row>
+    <row r="80" xml:space="preserve">
+      <c r="A80" t="str">
+        <v>SM-079</v>
+      </c>
+      <c r="B80" t="str">
+        <v>&gt;=2 bedrooms between ৳20,000-৳30,000</v>
+      </c>
+      <c r="C80" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D80" t="str">
+        <v>Combined EP — /search?bedrooms=2&amp;min_price=20000&amp;max_price=30000</v>
+      </c>
+      <c r="E80" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?bedrooms=2&amp;min_price=20000&amp;max_price=30000
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F80" t="str">
+        <v>2 rentals found</v>
+      </c>
+      <c r="G80" t="str">
+        <v/>
+      </c>
+      <c r="H80" t="str">
+        <v>Medium | ep | automated</v>
+      </c>
+    </row>
+    <row r="81" xml:space="preserve">
+      <c r="A81" t="str">
+        <v>SM-080</v>
+      </c>
+      <c r="B81" t="str">
+        <v>family flats, 4+ bedrooms</v>
+      </c>
+      <c r="C81" t="str">
+        <v>8 approved listings (live seed: rents ৳6,000–৳35,000)</v>
+      </c>
+      <c r="D81" t="str">
+        <v>Combined EP — /search?type[]=family&amp;bedrooms=4</v>
+      </c>
+      <c r="E81" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open /search?type[]=family&amp;bedrooms=4
+2. Read the 'N rentals found' counter</v>
+      </c>
+      <c r="F81" t="str">
+        <v>1 rental found</v>
+      </c>
+      <c r="G81" t="str">
+        <v/>
+      </c>
+      <c r="H81" t="str">
+        <v>Medium | ep | automated</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H81"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>